<commit_message>
Fix dedup in invetory_scope
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2505,11 +2505,11 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>["db02.dev"]</t>
+          <t>["db02.dev", "db02.staging"]</t>
         </is>
       </c>
       <c r="J6" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2585,11 +2585,11 @@
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal"]</t>
+          <t>["web01.prod.company.com", "web01.internal"]</t>
         </is>
       </c>
       <c r="J8" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -2625,11 +2625,11 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>["web02.external"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="J9" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -2665,11 +2665,11 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal"]</t>
+          <t>["web03.prod.internal", "web03.internal"]</t>
         </is>
       </c>
       <c r="J10" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3009,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3052,6 +3052,18 @@
           <t>Facts</t>
         </is>
       </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Host names before
+deduplication</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>Host names before
+deduplication count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
@@ -3082,6 +3094,14 @@
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
       </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>["app01.cluster"]</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -3112,6 +3132,14 @@
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
       </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>["app01.failover"]</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -3142,6 +3170,14 @@
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
       </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>["cache01.internal"]</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -3172,6 +3208,14 @@
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
       </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>["db01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -3180,67 +3224,83 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>45847.56953703704</v>
+        <v>45847.57300925926</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Development", "Staging"]</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Development Inventory", "Staging Inventory"]</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>["db02.dev", "db02.staging"]</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>db02.staging</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>45847.57300925926</v>
+        <v>45847.59069430155</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>["Staging"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>["Staging Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.staging"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
+          <t>{"ansible_connection_variable": ["tcp"]}</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>["log01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>45847.59069430155</v>
+        <v>45847.46905078303</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
@@ -3249,28 +3309,36 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"]}</t>
-        </is>
+          <t>{"ansible_connection_variable": ["ssh"]}</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>45847.45553240741</v>
+        <v>45847.68759259259</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
@@ -3279,28 +3347,36 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>["web02.external", "web02.internal"]</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>web01.prod.company.com</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>45847.46905078303</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
@@ -3314,67 +3390,83 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>["web03.internal", "web03.prod.internal"]</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>45847.68759259259</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>["web04.dev"]</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>web02.internal</t>
+          <t>web04.staging</t>
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Staging"]</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Staging Inventory"]</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.internal"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
@@ -3382,125 +3474,13 @@
           <t>{"ansible_connection_variable": ["ssh"]}</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>web03.internal</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="n">
-        <v>45847.75</v>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>["Production"]</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>["Production Inventory"]</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal"]}</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>web03.prod.internal</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="n">
-        <v>45847.75347222222</v>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>["Production"]</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>["Production Inventory"]</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.prod.internal"]}</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>web04.dev</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="n">
-        <v>45847.79166666666</v>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>["Development"]</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>["Development Inventory"]</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>web04.staging</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="n">
-        <v>45847.79513888889</v>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>["Staging"]</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>["Staging Inventory"]</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
-        </is>
-      </c>
-      <c r="F16" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>["web04.staging"]</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix current test failing on new column thatshould show only with dedup
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2585,7 +2585,7 @@
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>["web01.prod.company.com", "web01.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="J8" s="15" t="n">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["web02.internal", "web02.external"]</t>
         </is>
       </c>
       <c r="J9" s="15" t="n">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>["web03.prod.internal", "web03.internal"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="J10" s="15" t="n">

</xml_diff>

<commit_message>
Refactor host_names before dedup
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -3054,14 +3054,17 @@
       </c>
       <c r="G1" s="14" t="inlineStr">
         <is>
-          <t>Host names before
+          <t>Host names
+before
 deduplication</t>
         </is>
       </c>
       <c r="H1" s="14" t="inlineStr">
         <is>
-          <t>Host names before
-deduplication count</t>
+          <t>Host names
+before
+deduplication
+count</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add more test cases for deduplication
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -672,7 +672,7 @@
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr"/>
       <c r="G7" s="8" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="n">
@@ -1568,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1841,7 +1841,7 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Cache Management</t>
+          <t>AWS Instance Configuration</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -1850,28 +1850,28 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>45847.59739583333</v>
+        <v>45848.875</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>45847.59739583333</v>
+        <v>45848.87847222222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Cross-Org App Deploy</t>
+          <t>Cache Management</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1889,19 +1889,19 @@
         <v>1</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>45848.72222222222</v>
+        <v>45847.59739583333</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>45848.72222222222</v>
+        <v>45847.59739583333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Cross-Org Web Deploy</t>
+          <t>Cross-Org App Deploy</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -1919,19 +1919,19 @@
         <v>1</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>45847.45553240741</v>
+        <v>45848.72222222222</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>45847.45553240741</v>
+        <v>45848.72222222222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Database Backup</t>
+          <t>Cross-Org Web Deploy</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -1949,19 +1949,19 @@
         <v>1</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45847.45553240741</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45847.45553240741</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Deploy Web Application</t>
+          <t>Database Backup</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1976,22 +1976,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>45847.45207118545</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>45847.46898291037</v>
+        <v>45847.56672249403</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Log Management</t>
+          <t>Deploy Web Application</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -2006,22 +2006,22 @@
         <v>1</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.46898291037</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Multi-Node App</t>
+          <t>Log Management</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -2030,28 +2030,28 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>45848.70833333334</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>45848.72916666666</v>
+        <v>45847.59062642889</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Web Deployment</t>
+          <t>Multi-Node App</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -2063,25 +2063,25 @@
         <v>2</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45848.70833333334</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45848.72916666666</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Web03 Deploy</t>
+          <t>Remote Site Management</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -2090,28 +2090,28 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>45847.75</v>
+        <v>45848.91666666666</v>
       </c>
       <c r="H17" s="16" t="n">
-        <v>45847.75</v>
+        <v>45848.92013888889</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Web03 Prod Deploy</t>
+          <t>Web Deployment</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -2120,33 +2120,33 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G18" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.6875</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Staging Database Setup</t>
+          <t>Web03 Deploy</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
@@ -2159,24 +2159,24 @@
         <v>1</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.75</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.75</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Staging Multi-Node App</t>
+          <t>Web03 Prod Deploy</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
@@ -2189,42 +2189,132 @@
         <v>1</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G20" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="H20" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45847.75347222222</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
+          <t>Windows Patching</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>45848.83680555555</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Staging Database Setup</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Staging Multi-Node App</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
           <t>Web04 Staging Deploy</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="C21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="15" t="n">
+      <c r="C24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="G21" s="16" t="n">
+      <c r="G24" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="H21" s="16" t="n">
+      <c r="H24" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
     </row>
@@ -2239,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2315,37 +2405,37 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>app01.cluster</t>
+          <t>203.0.113.10</t>
         </is>
       </c>
       <c r="B2" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>45848.70833333334</v>
+        <v>45848.91666666666</v>
       </c>
       <c r="F2" s="16" t="n">
-        <v>45848.72222222222</v>
+        <v>45848.92013888889</v>
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["nat-shared-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "internal_ip": ["10.0.1.10", "10.0.1.11"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
-          <t>["app01.cluster"]</t>
+          <t>["203.0.113.10"]</t>
         </is>
       </c>
       <c r="J2" s="15" t="n">
@@ -2355,37 +2445,37 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>app01.failover</t>
+          <t>app01.cluster</t>
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>45848.72916666666</v>
+        <v>45848.70833333334</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>45848.72916666666</v>
+        <v>45848.72222222222</v>
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>["app01.failover"]</t>
+          <t>["app01.cluster"]</t>
         </is>
       </c>
       <c r="J3" s="15" t="n">
@@ -2395,37 +2485,37 @@
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>cache01.internal</t>
+          <t>app01.failover</t>
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>45847.59739583333</v>
+        <v>45848.72916666666</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>45847.60086805555</v>
+        <v>45848.72916666666</v>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>["cache01.internal"]</t>
+          <t>["app01.failover"]</t>
         </is>
       </c>
       <c r="J4" s="15" t="n">
@@ -2435,47 +2525,47 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>db01.company.com</t>
+          <t>aws-vm-01.us-east</t>
         </is>
       </c>
       <c r="B5" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45848.875</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45848.87847222222</v>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>["db01.company.com"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
         </is>
       </c>
       <c r="J5" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>db02.dev</t>
+          <t>cache01.internal</t>
         </is>
       </c>
       <c r="B6" s="15" t="n">
@@ -2485,37 +2575,37 @@
         <v>2</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>45847.56949074074</v>
+        <v>45847.59739583333</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.60086805555</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>["db02.dev", "db02.staging"]</t>
+          <t>["cache01.internal"]</t>
         </is>
       </c>
       <c r="J6" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>db01.company.com</t>
         </is>
       </c>
       <c r="B7" s="15" t="n">
@@ -2525,27 +2615,27 @@
         <v>1</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["db01.company.com"]</t>
         </is>
       </c>
       <c r="J7" s="15" t="n">
@@ -2555,37 +2645,37 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>db02.dev</t>
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>45847.45207118545</v>
+        <v>45847.56949074074</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>45847.46898291037</v>
+        <v>45847.57296296296</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["db02.dev", "db02.staging"]</t>
         </is>
       </c>
       <c r="J8" s="15" t="n">
@@ -2595,77 +2685,77 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="J9" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>45847.75</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.46898291037</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="J10" s="15" t="n">
@@ -2675,80 +2765,240 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.6875</v>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="J11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
+          <t>web03.internal</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>45847.75</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>["web03.internal", "web03.prod.internal"]</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>web04.dev</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>["web04.dev"]</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
           <t>web04.staging</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="15" t="n">
+      <c r="B14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E14" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F14" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
-      <c r="H12" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
         <is>
           <t>["web04.staging"]</t>
         </is>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J14" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="J15" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>win-srv02.company.com</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>45848.83680555555</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>45848.83680555555</v>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv02.company.com"]</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3009,7 +3259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3071,35 +3321,35 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>app01.cluster</t>
+          <t>203.0.113.10</t>
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>45847.72239583333</v>
+        <v>45846.92013888889</v>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Production", "Staging"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Development Inventory", "Production Inventory", "Staging Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["nat-shared-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "internal_ip": ["10.0.1.10", "10.0.1.11"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>["app01.cluster"]</t>
+          <t>["203.0.113.10"]</t>
         </is>
       </c>
       <c r="H2" s="15" t="n">
@@ -3109,35 +3359,35 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>app01.failover</t>
+          <t>app01.cluster</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>45847.72930555556</v>
+        <v>45847.72239583333</v>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development", "Production", "Staging"]</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Development Inventory", "Production Inventory", "Staging Inventory"]</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>["app01.failover"]</t>
+          <t>["app01.cluster"]</t>
         </is>
       </c>
       <c r="H3" s="15" t="n">
@@ -3147,35 +3397,35 @@
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>cache01.internal</t>
+          <t>app01.failover</t>
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>45847.60104166667</v>
+        <v>45847.72930555556</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Production"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>["cache01.internal"]</t>
+          <t>["app01.failover"]</t>
         </is>
       </c>
       <c r="H4" s="15" t="n">
@@ -3185,11 +3435,11 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>db01.company.com</t>
+          <t>aws-vm-01.us-east</t>
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>45847.56676651941</v>
+        <v>45846.87847222222</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
@@ -3203,69 +3453,69 @@
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>["db01.company.com"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
         </is>
       </c>
       <c r="H5" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>db02.dev</t>
+          <t>cache01.internal</t>
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>45847.57300925926</v>
+        <v>45847.60104166667</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Staging"]</t>
+          <t>["Development", "Production"]</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory", "Staging Inventory"]</t>
+          <t>["Development Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>["db02.dev", "db02.staging"]</t>
+          <t>["cache01.internal"]</t>
         </is>
       </c>
       <c r="H6" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>db01.company.com</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>45847.59069430155</v>
+        <v>45847.56676651941</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
@@ -3279,17 +3529,17 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["db01.company.com"]</t>
         </is>
       </c>
       <c r="H7" s="15" t="n">
@@ -3299,35 +3549,35 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>db02.dev</t>
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>45847.46905078303</v>
+        <v>45847.57300925926</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development", "Staging"]</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Production Inventory"]</t>
+          <t>["Development Inventory", "Staging Inventory"]</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["db02.dev", "db02.staging"]</t>
         </is>
       </c>
       <c r="H8" s="15" t="n">
@@ -3337,11 +3587,11 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>45847.68759259259</v>
+        <v>45847.59069430155</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
@@ -3355,31 +3605,31 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="H9" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.46905078303</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
@@ -3388,22 +3638,22 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="H10" s="15" t="n">
@@ -3413,76 +3663,228 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.68759259259</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="H11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
+          <t>web03.internal</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>["web03.internal", "web03.prod.internal"]</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>web04.dev</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>["Development"]</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>["Development Inventory"]</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>["web04.dev"]</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
           <t>web04.staging</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B14" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>["Staging"]</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>["Staging Inventory"]</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["ssh"]}</t>
-        </is>
-      </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>["web04.staging"]</t>
         </is>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H14" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>45846.83333333334</v>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>win-srv02.company.com</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>45846.83680555555</v>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv02.company.com"]</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3607,13 +4009,13 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C4" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C4" s="15" t="n">
-        <v>8</v>
-      </c>
       <c r="D4" s="15" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0</v>
@@ -3622,7 +4024,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>97</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Fix some failing tests
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -84,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffcc17"/>
+        <fgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,7 +160,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -672,7 +671,7 @@
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr"/>
       <c r="G7" s="8" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="n">
@@ -778,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -819,19 +818,19 @@
         </is>
       </c>
       <c r="B2" s="17" t="n">
-        <v>45847.99998842592</v>
+        <v>45848.99998842592</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>45848.04215277778</v>
+        <v>45850</v>
       </c>
       <c r="D2" t="n">
-        <v>3643</v>
+        <v>86401</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>job_host_summary.csv</t>
+          <t>main_host.csv</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
@@ -847,7 +846,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>main_host.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="B4" s="17" t="n">
@@ -860,63 +859,72 @@
         <v>86401</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>main_indirectmanagednodeaudit.csv</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="n">
-        <v>45848.99998842592</v>
-      </c>
-      <c r="C5" s="17" t="n">
-        <v>45850</v>
-      </c>
-      <c r="D5" t="n">
-        <v>86401</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Collection timestamp</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Filter since</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Filter until</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>CSV filename</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Elapsed</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Time since
 previous collection</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="17" t="n"/>
+    </row>
     <row r="8">
       <c r="A8" s="17" t="n">
-        <v>45846.99998842592</v>
+        <v>45846</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>45846</v>
@@ -926,7 +934,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>job_host_summary.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -937,11 +945,13 @@
       <c r="F8" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="17" t="n"/>
+      <c r="G8" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="n">
-        <v>45846.99998842592</v>
+        <v>45846</v>
       </c>
       <c r="B9" s="17" t="n">
         <v>45846</v>
@@ -951,7 +961,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>main_host.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -962,11 +972,13 @@
       <c r="F9" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="17" t="n"/>
+      <c r="G9" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="n">
-        <v>45846.99998842592</v>
+        <v>45846</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>45846</v>
@@ -987,21 +999,23 @@
       <c r="F10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="17" t="n"/>
+      <c r="G10" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="B11" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>45847.99998842592</v>
+        <v>45846.99998842592</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>job_host_summary.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1013,22 +1027,22 @@
         <v>0</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>1.157407407407407e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="B12" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>45847.99998842592</v>
+        <v>45846.99998842592</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>main_host.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1040,18 +1054,18 @@
         <v>0</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>1.157407407407407e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="B13" s="17" t="n">
-        <v>45847</v>
+        <v>45846</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>45847.99998842592</v>
+        <v>45846.99998842592</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1066,19 +1080,17 @@
       <c r="F13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="18" t="n">
-        <v>1.157407407407407e-05</v>
-      </c>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="17" t="n">
-        <v>45848</v>
+        <v>45846</v>
       </c>
       <c r="B14" s="17" t="n">
-        <v>45848</v>
+        <v>45846</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>45848.99998842592</v>
+        <v>45846.99998842592</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1094,22 +1106,22 @@
         <v>0</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="n">
-        <v>45848</v>
+        <v>45846</v>
       </c>
       <c r="B15" s="17" t="n">
-        <v>45848</v>
+        <v>45846</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>45848.99998842592</v>
+        <v>45846.99998842592</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>main_indirectmanagednodeaudit.csv</t>
+          <t>main_host.csv</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1121,37 +1133,656 @@
         <v>0</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="17" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="n">
+        <v>45846.00001157408</v>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <v>1.157407407407407e-05</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="n">
+        <v>45846.00002314815</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <v>45846</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>45846.99998842592</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>main_indirectmanagednodeaudit.csv</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>2.314814814814815e-05</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B23" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>45847.00001157408</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>45847.00002314815</v>
+      </c>
+      <c r="B30" s="17" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>45847.99998842592</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>main_indirectmanagednodeaudit.csv</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C31" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C32" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B35" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B36" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>job_host_summary.csv</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n">
+        <v>45848.00001157408</v>
+      </c>
+      <c r="B37" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>main_host.csv</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n">
+        <v>45848.00002314815</v>
+      </c>
+      <c r="B38" s="17" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>45848.99998842592</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>main_indirectmanagednodeaudit.csv</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n">
         <v>45848.04215277778</v>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B39" s="17" t="n">
         <v>45848.04215277778</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C39" s="17" t="n">
         <v>45848.99998842592</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>job_host_summary.csv</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="19" t="n">
-        <v>1.042152777777778</v>
-      </c>
-    </row>
-    <row r="17"/>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="18" t="n">
+        <v>0.04215277777777778</v>
+      </c>
+    </row>
+    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1163,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1226,12 +1857,12 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Database Job</t>
+          <t>Kubernetes Template</t>
         </is>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
@@ -1244,46 +1875,54 @@
         <v>1</v>
       </c>
       <c r="F2" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>45846.41666666666</v>
+      </c>
+      <c r="H2" s="16" t="n">
+        <v>45846.41666666666</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Dev Deploy</t>
+          <t>VMware Template</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E3" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>45846.3905170645</v>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>45846.3905170645</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Dev Setup</t>
+          <t>VMware_Template2</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
@@ -1298,18 +1937,22 @@
       <c r="F4" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
+      <c r="G4" s="16" t="n">
+        <v>45846.4042064301</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>45846.4042064301</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Backup Job</t>
+          <t>Dev Cache Management</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Disaster Recovery</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
@@ -1322,20 +1965,24 @@
         <v>1</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>45847.60086805555</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>45847.60086805555</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>Monitoring Job</t>
+          <t>Dev Database Setup</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
@@ -1348,67 +1995,79 @@
         <v>1</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>45847.56949074074</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>45847.56949074074</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Cache Update Job</t>
+          <t>Dev Multi-Node App</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>45848.71180555555</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>45848.71180555555</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Cloud Deploy</t>
+          <t>Web04 Dev Deploy</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Database Job</t>
+          <t>API Server Deploy</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -1417,24 +2076,28 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>45846.54166666666</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>45846.54861111111</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Log Collection</t>
+          <t>AWS Instance Configuration</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1443,24 +2106,28 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
+        <v>24</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>45848.875</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>45848.87847222222</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Network Config</t>
+          <t>Cache Management</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -1469,24 +2136,28 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>45847.59739583333</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>45847.59739583333</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Production Job</t>
+          <t>Cross-Org App Deploy</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -1495,24 +2166,28 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>65</v>
-      </c>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>45848.72222222222</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>45848.72222222222</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Windows Update</t>
+          <t>Cross-Org Web Deploy</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1521,29 +2196,33 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>45847.45553240741</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>45847.45553240741</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>QA Test Job</t>
+          <t>Database Backup</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>QA Team</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
@@ -1556,50 +2235,58 @@
         <v>1</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>45847.56672249403</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>45847.56672249403</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Database Job</t>
+          <t>Database Primary Deploy</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="16" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>45846.58333333334</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>45846.59027777778</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Staging Deploy</t>
+          <t>Deploy Web Application</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>1</v>
@@ -1608,10 +2295,314 @@
         <v>2</v>
       </c>
       <c r="F16" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="G16" s="16" t="n">
+        <v>45847.45207118545</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>45847.46898291037</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Log Management</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
+      <c r="G17" s="16" t="n">
+        <v>45847.59062642889</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>45847.59062642889</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Multi-Node App</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G18" s="16" t="n">
+        <v>45848.70833333334</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>45848.72916666666</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Remote Site Management</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>45848.91666666666</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>45848.92013888889</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Web Deployment</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>45847.66666666666</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>45847.6875</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Web03 Deploy</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>45847.75</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>45847.75</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Web03 Prod Deploy</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Windows Patching</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>45848.83680555555</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Staging Database Setup</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Staging Multi-Node App</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Web04 Staging Deploy</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>45847.79513888889</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>45847.79513888889</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1624,7 +2615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1700,37 +2691,37 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>app01.cluster</t>
+          <t>203.0.113.10</t>
         </is>
       </c>
       <c r="B2" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>45846.41666666666</v>
+        <v>45848.91666666666</v>
       </c>
       <c r="F2" s="16" t="n">
-        <v>45848.41666666666</v>
+        <v>45848.92013888889</v>
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["nat-shared-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "internal_ip": ["10.0.1.10", "10.0.1.11"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
-          <t>["app01.cluster"]</t>
+          <t>["203.0.113.10"]</t>
         </is>
       </c>
       <c r="J2" s="15" t="n">
@@ -1740,27 +2731,27 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>app01.failover</t>
+          <t>api-server</t>
         </is>
       </c>
       <c r="B3" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>45846.4375</v>
+        <v>45846.54166666666</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>45848.4375</v>
+        <v>45846.54861111111</v>
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["api-server-001"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL360-API"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
@@ -1770,57 +2761,57 @@
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>["app01.failover"]</t>
+          <t>["api-server", "api-server.company.com", "api-server.company.com.east"]</t>
         </is>
       </c>
       <c r="J3" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>aws-vm-01.us-east</t>
+          <t>app01.cluster</t>
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="15" t="n">
         <v>4</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>45846.77083333334</v>
+        <v>45848.70833333334</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>45847.58333333334</v>
+        <v>45848.72222222222</v>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
+          <t>["app01.cluster"]</t>
         </is>
       </c>
       <c r="J4" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>backup-srv-01.dr</t>
+          <t>app01.failover</t>
         </is>
       </c>
       <c r="B5" s="15" t="n">
@@ -1830,27 +2821,27 @@
         <v>1</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>45848.5625</v>
+        <v>45848.72916666666</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>45848.5625</v>
+        <v>45848.72916666666</v>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["backup-srv-01.dr"], "ansible_machine_id": ["backup-dr-001"], "ansible_port": [22], "ansible_product_serial": ["DR-BACKUP-001"], "host_name": ["backup-srv-01.dr"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>["backup-srv-01.dr"]</t>
+          <t>["app01.failover"]</t>
         </is>
       </c>
       <c r="J5" s="15" t="n">
@@ -1860,7 +2851,7 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>cache01.internal</t>
+          <t>aws-vm-01.us-east</t>
         </is>
       </c>
       <c r="B6" s="15" t="n">
@@ -1870,67 +2861,67 @@
         <v>2</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>45846.45833333334</v>
+        <v>45848.875</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>45847.4375</v>
+        <v>45848.87847222222</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>["cache01.internal"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
         </is>
       </c>
       <c r="J6" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>db01.company.com</t>
+          <t>cache01.internal</t>
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="15" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>45846.47916666666</v>
+        <v>45847.59739583333</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>45847.45833333334</v>
+        <v>45847.60086805555</v>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>["db01.company.com"]</t>
+          <t>["cache01.internal"]</t>
         </is>
       </c>
       <c r="J7" s="15" t="n">
@@ -1940,47 +2931,47 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>db02.dev</t>
+          <t>db-primary</t>
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>45846.5</v>
+        <v>45846.58333333334</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>45847.60416666666</v>
+        <v>45846.58333333334</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["db-primary-001"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750-DB"], "host_name": ["db-primary"]}</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>["db02.dev", "db02.staging"]</t>
+          <t>["db-primary"]</t>
         </is>
       </c>
       <c r="J8" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>db-primary.company.com</t>
         </is>
       </c>
       <c r="B9" s="15" t="n">
@@ -1990,27 +2981,27 @@
         <v>1</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>45846.54166666666</v>
+        <v>45846.58680555555</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>45846.54166666666</v>
+        <v>45846.58680555555</v>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["db-primary.company.com"], "ansible_port": [22], "host_name": ["db-primary.company.com"]}</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["db-primary.company.com"]</t>
         </is>
       </c>
       <c r="J9" s="15" t="n">
@@ -2020,7 +3011,7 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>mobile-dev-laptop.office.company.com</t>
+          <t>db-primary.company.com.west</t>
         </is>
       </c>
       <c r="B10" s="15" t="n">
@@ -2030,27 +3021,27 @@
         <v>1</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>45846.85416666666</v>
+        <v>45846.59027777778</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>45846.85416666666</v>
+        <v>45846.59027777778</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["mobile-laptop-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-LAPTOP-XPS13-001"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
+          <t>{"ansible_host": ["db-primary.company.com.west"], "ansible_port": [22], "host_name": ["db-primary.company.com.west"]}</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>["mobile-dev-laptop.office.company.com"]</t>
+          <t>["db-primary.company.com.west"]</t>
         </is>
       </c>
       <c r="J10" s="15" t="n">
@@ -2060,7 +3051,7 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>monitor-01.ops</t>
+          <t>db01.company.com</t>
         </is>
       </c>
       <c r="B11" s="15" t="n">
@@ -2070,27 +3061,27 @@
         <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>45848.54166666666</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>45848.54166666666</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["monitor-01.ops"], "ansible_machine_id": ["monitor-ops-001"], "ansible_port": [22], "ansible_product_serial": ["OPS-MONITOR-001"], "host_name": ["monitor-01.ops"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>["monitor-01.ops"]</t>
+          <t>["db01.company.com"]</t>
         </is>
       </c>
       <c r="J11" s="15" t="n">
@@ -2100,47 +3091,47 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>nat-host-01.external</t>
+          <t>db02.dev</t>
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="15" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>45846.8125</v>
+        <v>45847.56949074074</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>45847.5625</v>
+        <v>45847.57296296296</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>["nat-host-01.external"]</t>
+          <t>["db02.dev", "db02.staging"]</t>
         </is>
       </c>
       <c r="J12" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>nat-host-02.external</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B13" s="15" t="n">
@@ -2150,27 +3141,27 @@
         <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>45846.83333333334</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>45846.83333333334</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>["nat-host-02.external"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="J13" s="15" t="n">
@@ -2180,67 +3171,67 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>test-host-01.qa</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>45848.52083333334</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>45848.52083333334</v>
+        <v>45847.46898291037</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["test-host-01.qa"], "ansible_machine_id": ["qa-test-001"], "ansible_port": [22], "ansible_product_serial": ["QA-TEST-SERVER-001"], "host_name": ["test-host-01.qa"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>["test-host-01.qa"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="J14" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>45846.5625</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>45847.625</v>
+        <v>45847.6875</v>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -2250,7 +3241,7 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="J15" s="15" t="n">
@@ -2260,27 +3251,27 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>45846.60416666666</v>
+        <v>45847.75</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>45847.5</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -2290,7 +3281,7 @@
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="J16" s="15" t="n">
@@ -2300,27 +3291,27 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>45846.64583333334</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>45847.52083333334</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -2330,37 +3321,37 @@
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web04.dev"]</t>
         </is>
       </c>
       <c r="J17" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web04.staging</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>45846.6875</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>45848.45833333334</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -2370,7 +3361,7 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web04.staging"]</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
@@ -2380,37 +3371,37 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>win-srv01.company.com</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>45846.70833333334</v>
+        <v>45848.83333333334</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>45848.47916666666</v>
+        <v>45848.83333333334</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["win-srv01.company.com"]</t>
         </is>
       </c>
       <c r="J19" s="15" t="n">
@@ -2420,27 +3411,27 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>win-srv02.company.com</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>45846.72916666666</v>
+        <v>45848.83680555555</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>45848.5</v>
+        <v>45848.83680555555</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
@@ -2450,50 +3441,10 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["win-srv02.company.com"]</t>
         </is>
       </c>
       <c r="J20" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>win-srv02.company.com</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="16" t="n">
-        <v>45846.75</v>
-      </c>
-      <c r="F21" s="16" t="n">
-        <v>45846.75</v>
-      </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="inlineStr">
-        <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
-        </is>
-      </c>
-      <c r="I21" s="15" t="inlineStr">
-        <is>
-          <t>["win-srv02.company.com"]</t>
-        </is>
-      </c>
-      <c r="J21" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2508,7 +3459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2593,6 +3544,156 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>k8s-worker-01.internal</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>45846.41678240741</v>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>45846.41678240741</v>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_kubernetes_node_id": ["node-12345"], "ansible_port": [22]}</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>{"platform": ["kubernetes"]}</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>["INDIRECT"]</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>["k8s-worker-01.internal"]</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>vcenter-vm-01.internal</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>45846.39805042704</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>45846.39805042704</v>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_port": [22], "ansible_vmware_bios_uuid": ["420b1367-1e11-c9d7-4d0f-c3b3cba9ae16"], "ansible_vmware_instance_uuid": ["500b3d2e-9abe-8ee1-98ea-bf67b591c104"], "ansible_vmware_moid": ["vm-87212"]}</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>{"device_type": ["VM"]}</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>["INDIRECT"]</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>["vcenter-vm-01.internal"]</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>vcenter-vm-02.internal</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>45846.40586975554</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>45846.40586975554</v>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_port": [443], "ansible_vmware_bios_uuid": ["420ba1d2-3793-215c-30f0-5957a405d4e6"], "ansible_vmware_instance_uuid": ["500b1a63-d55d-bf21-c104-1617888dd7d2"], "ansible_vmware_moid": ["vm-87213"]}</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>{"device_type": ["VM"]}</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>["INDIRECT"]</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>["vcenter-vm-02.internal"]</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2604,7 +3705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2704,25 +3805,25 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>app01.cluster</t>
+          <t>api-server</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>45848.72239583333</v>
+        <v>45846.54861111111</v>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Production", "Staging"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Development Inventory", "Production Inventory", "Staging Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["api-server-001"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL360-API"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
@@ -2732,35 +3833,35 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>["app01.cluster"]</t>
+          <t>["api-server", "api-server.company.com", "api-server.company.com.east"]</t>
         </is>
       </c>
       <c r="H3" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>app01.failover</t>
+          <t>app01.cluster</t>
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>45848.72930555556</v>
+        <v>45847.72239583333</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development", "Production", "Staging"]</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Development Inventory", "Production Inventory", "Staging Inventory"]</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -2770,7 +3871,7 @@
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>["app01.failover"]</t>
+          <t>["app01.cluster"]</t>
         </is>
       </c>
       <c r="H4" s="15" t="n">
@@ -2780,11 +3881,11 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>aws-vm-01.us-east</t>
+          <t>app01.failover</t>
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>45846.87847222222</v>
+        <v>45847.72930555556</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
@@ -2798,59 +3899,59 @@
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
+          <t>["app01.failover"]</t>
         </is>
       </c>
       <c r="H5" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>backup-srv-01.dr</t>
+          <t>aws-vm-01.us-east</t>
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>45848.5625</v>
+        <v>45846.87847222222</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>["Disaster Recovery"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>["DR Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["backup-srv-01.dr"], "ansible_machine_id": ["backup-dr-001"], "ansible_port": [22], "ansible_product_serial": ["DR-BACKUP-001"], "host_name": ["backup-srv-01.dr"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>["backup-srv-01.dr"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
         </is>
       </c>
       <c r="H6" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2860,7 +3961,7 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>45848.60104166667</v>
+        <v>45847.60104166667</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
@@ -2894,11 +3995,11 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>db01.company.com</t>
+          <t>db-cluster-node1.internal</t>
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>45848.56676651941</v>
+        <v>45846.45833333334</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
@@ -2912,17 +4013,17 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["db-cluster-node1.internal"], "ansible_machine_id": ["db-node-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R750-DB-001"], "host_name": ["db-cluster-node1.internal"]}</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>["db01.company.com"]</t>
+          <t>["db-cluster-node1.internal"]</t>
         </is>
       </c>
       <c r="H8" s="15" t="n">
@@ -2932,49 +4033,49 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>db02.dev</t>
+          <t>db-cluster-node2.internal</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>45848.56953703704</v>
+        <v>45846.46180555555</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Staging"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory", "Staging Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["db-cluster-node2.internal"], "ansible_machine_id": ["db-node-002"], "ansible_port": [22], "ansible_product_serial": ["DELL-R750-DB-002"], "host_name": ["db-cluster-node2.internal"]}</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["secondary"]}</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>["db02.dev", "db02.staging"]</t>
+          <t>["db-cluster-node2.internal"]</t>
         </is>
       </c>
       <c r="H9" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>legacy01.old</t>
+          <t>db-primary</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>45848.66344907408</v>
+        <v>45846.58333333334</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
@@ -2988,17 +4089,17 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["legacy01.old"], "host_name": ["legacy01.old"]}</t>
+          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["db-primary-001"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750-DB"], "host_name": ["db-primary"]}</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>["legacy01.old"]</t>
+          <t>["db-primary"]</t>
         </is>
       </c>
       <c r="H10" s="15" t="n">
@@ -3008,11 +4109,11 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>db-primary.company.com</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>45847.59069430155</v>
+        <v>45846.58680555555</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
@@ -3026,17 +4127,17 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["db-primary.company.com"], "ansible_port": [22], "host_name": ["db-primary.company.com"]}</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["db-primary.company.com"]</t>
         </is>
       </c>
       <c r="H11" s="15" t="n">
@@ -3046,35 +4147,35 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>mobile-dev-laptop.office.company.com</t>
+          <t>db-primary.company.com.west</t>
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>45846.375</v>
+        <v>45846.59027777778</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["mobile-laptop-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-LAPTOP-XPS13-001"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
+          <t>{"ansible_host": ["db-primary.company.com.west"], "ansible_port": [22], "host_name": ["db-primary.company.com.west"]}</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>["mobile-dev-laptop.office.company.com"]</t>
+          <t>["db-primary.company.com.west"]</t>
         </is>
       </c>
       <c r="H12" s="15" t="n">
@@ -3084,35 +4185,35 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>monitor-01.ops</t>
+          <t>db01.company.com</t>
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>45848.54166666666</v>
+        <v>45847.56676651941</v>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>["Operations"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>["Operations Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["monitor-01.ops"], "ansible_machine_id": ["monitor-ops-001"], "ansible_port": [22], "ansible_product_serial": ["OPS-MONITOR-001"], "host_name": ["monitor-01.ops"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>["monitor-01.ops"]</t>
+          <t>["db01.company.com"]</t>
         </is>
       </c>
       <c r="H13" s="15" t="n">
@@ -3122,73 +4223,73 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>test-host-01.qa</t>
+          <t>db02.dev</t>
         </is>
       </c>
       <c r="B14" s="16" t="n">
-        <v>45848.52083333334</v>
+        <v>45847.57300925926</v>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>["QA Team"]</t>
+          <t>["Development", "Staging"]</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>["QA Inventory"]</t>
+          <t>["Development Inventory", "Staging Inventory"]</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["test-host-01.qa"], "ansible_machine_id": ["qa-test-001"], "ansible_port": [22], "ansible_product_serial": ["QA-TEST-SERVER-001"], "host_name": ["test-host-01.qa"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>["test-host-01.qa"]</t>
+          <t>["db02.dev", "db02.staging"]</t>
         </is>
       </c>
       <c r="H14" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>web01.example.com</t>
+          <t>legacy-server.company.com</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>45848.51093892889</v>
+        <v>45846.50347222222</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development", "Production"]</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Development Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.example.com"], "ansible_machine_id": ["abc123"], "ansible_port": ["ssh"], "ansible_product_serial": ["HP-ProLiant-DL360"], "host_name": ["web01.example.com"]}</t>
+          <t>{"ansible_machine_id": ["legacy-001"], "ansible_port": [22], "ansible_product_serial": ["HP-DL380-LEGACY-001"], "host_name": ["legacy-server.company.com"], "ansible_host": ["legacy-server.company.com"]}</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "server_type": ["legacy"]}</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>["web01.example.com"]</t>
+          <t>["legacy-server.company.com"]</t>
         </is>
       </c>
       <c r="H15" s="15" t="n">
@@ -3198,11 +4299,11 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B16" s="16" t="n">
-        <v>45847.46905078303</v>
+        <v>45847.59069430155</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
@@ -3211,36 +4312,36 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="H16" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>web02.dev</t>
+          <t>mobile-dev-laptop.office.company.com</t>
         </is>
       </c>
       <c r="B17" s="16" t="n">
-        <v>45848.51440972222</v>
+        <v>45846.375</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
@@ -3254,17 +4355,17 @@
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.dev"], "ansible_machine_id": ["def456"], "ansible_port": ["ssh"], "ansible_product_serial": ["HP-ProLiant-DL360"], "host_name": ["web02.dev"]}</t>
+          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["mobile-laptop-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-LAPTOP-XPS13-001"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>["web02.dev"]</t>
+          <t>["mobile-dev-laptop.office.company.com"]</t>
         </is>
       </c>
       <c r="H17" s="15" t="n">
@@ -3274,11 +4375,11 @@
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>45847.68759259259</v>
+        <v>45847.46905078303</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
@@ -3287,12 +4388,12 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
@@ -3302,7 +4403,7 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="H18" s="15" t="n">
@@ -3312,11 +4413,11 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B19" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.68759259259</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
@@ -3330,7 +4431,7 @@
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
@@ -3340,7 +4441,7 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="H19" s="15" t="n">
@@ -3350,25 +4451,25 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B20" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -3378,35 +4479,35 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="H20" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>["Staging"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>["Staging Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
@@ -3416,7 +4517,7 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["web04.dev"]</t>
         </is>
       </c>
       <c r="H21" s="15" t="n">
@@ -3426,35 +4527,35 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>web04.staging</t>
         </is>
       </c>
       <c r="B22" s="16" t="n">
-        <v>45846.83333333334</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Staging"]</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Staging Inventory"]</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["web04.staging"]</t>
         </is>
       </c>
       <c r="H22" s="15" t="n">
@@ -3464,38 +4565,114 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
+          <t>webserver.company.com</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="n">
+        <v>45846.42013888889</v>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["web-backup-001", "web-primary-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-WEB-001", "DELL-R740-WEB-002"], "host_name": ["webserver.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "server_role": ["backup", "primary"]}</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>["webserver.company.com"]</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>45846.83333333334</v>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
           <t>win-srv02.company.com</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B25" s="16" t="n">
         <v>45846.83680555555</v>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>["Production"]</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>["Production Inventory"]</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="G25" s="15" t="inlineStr">
         <is>
           <t>["win-srv02.company.com"]</t>
         </is>
       </c>
-      <c r="H23" s="15" t="n">
+      <c r="H25" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3510,7 +4687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3566,42 +4743,42 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="B2" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="15" t="n">
-        <v>0</v>
-      </c>
       <c r="F2" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G2" s="15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Disaster Recovery</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0</v>
@@ -3610,23 +4787,23 @@
         <v>0</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0</v>
@@ -3635,23 +4812,23 @@
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>4</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Staging</t>
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>0</v>
@@ -3660,57 +4837,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>QA Team</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="15" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Staging</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="15" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -3724,7 +4851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3766,6 +4893,25 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>ansible.builtin</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="15" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3777,7 +4923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3819,6 +4965,25 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>No role used</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="15" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3830,7 +4995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3872,6 +5037,44 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>ansible.builtin.debug</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="15" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>ansible.builtin.setup</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
More cleanup of the tests and regenerated data
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2716,7 +2716,7 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "internal_ip": ["10.0.1.10", "10.0.1.11"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "internal_ip": ["10.0.1.10", "10.0.1.11"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix failures of data_statuses assert
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1644,12 +1644,12 @@
         <v>0</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="n">
-        <v>45848</v>
+        <v>45848.00001157408</v>
       </c>
       <c r="B35" s="17" t="n">
         <v>45848</v>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>job_host_summary.csv</t>
+          <t>main_host.csv</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1671,12 +1671,12 @@
         <v>0</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="n">
-        <v>45848</v>
+        <v>45848.00002314815</v>
       </c>
       <c r="B36" s="17" t="n">
         <v>45848</v>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>job_host_summary.csv</t>
+          <t>main_indirectmanagednodeaudit.csv</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1698,22 +1698,22 @@
         <v>0</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="n">
-        <v>45848.00001157408</v>
+        <v>45848.04215277778</v>
       </c>
       <c r="B37" s="17" t="n">
-        <v>45848</v>
+        <v>45848.04215277778</v>
       </c>
       <c r="C37" s="17" t="n">
         <v>45848.99998842592</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>main_host.csv</t>
+          <t>job_host_summary.csv</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1725,22 +1725,22 @@
         <v>0</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="n">
-        <v>45848.00002314815</v>
+        <v>45848.04215277778</v>
       </c>
       <c r="B38" s="17" t="n">
-        <v>45848</v>
+        <v>45848.04215277778</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>45848.99998842592</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>main_indirectmanagednodeaudit.csv</t>
+          <t>job_host_summary.csv</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1752,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>1</v>
+        <v>0.04215277777777778</v>
       </c>
     </row>
     <row r="39">
@@ -1779,7 +1779,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.04215277777777778</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40"/>

</xml_diff>

<commit_message>
Add more facts into collection
Will help to debug deduplication issues
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2716,7 +2716,7 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["OptiPlex 7090"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Core(TM) i7-10700 CPU @ 2.90GHz"], "ansible_form_factor": ["Desktop"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["1.2.3"], "ansible_board_serial": ["NAT-GW-001", "NAT-GW-002"]}</t>
         </is>
       </c>
       <c r="I2" s="15" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL360 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U32"], "ansible_board_serial": ["API-SERVER-001"]}</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL380 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U30"], "ansible_board_serial": ["USE1234567"]}</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL380 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U30"], "ansible_board_serial": ["USE7654321"]}</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Amazon EC2"], "ansible_product_name": ["m5.large"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Platinum 8259CL CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Amazon EC2"], "ansible_bios_version": ["1.0"], "ansible_board_serial": ["ec2-instance"]}</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"]}</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["AMD EPYC 7542 32-Core Processor"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.14.0"], "ansible_board_serial": ["DB-PRIMARY-001"]}</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A86"]}</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A87"]}</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["OptiPlex 7090"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Core(TM) i7-10700 CPU @ 2.90GHz"], "ansible_form_factor": ["Desktop"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["1.2.3"], "ansible_board_serial": ["NAT-GW-001", "NAT-GW-002"]}</t>
         </is>
       </c>
       <c r="G2" s="15" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL360 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U32"], "ansible_board_serial": ["API-SERVER-001"]}</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL380 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U30"], "ansible_board_serial": ["USE1234567"]}</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL380 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U30"], "ansible_board_serial": ["USE7654321"]}</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "aws_instance_id": ["i-0a1b2c3d4e5f6g7h8", "i-9z8y7x6w5v4u3t2s"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Amazon EC2"], "ansible_product_name": ["m5.large"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Platinum 8259CL CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Amazon EC2"], "ansible_bios_version": ["1.0"], "ansible_board_serial": ["ec2-instance"]}</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"]}</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["AMD EPYC 7542 32-Core Processor"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.14.0"], "ansible_board_serial": ["DB-PRIMARY-001"]}</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A86"]}</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["xen"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A87"]}</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["XPS 13 9310"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Core(TM) i7-1165G7 CPU @ 2.80GHz"], "ansible_form_factor": ["Laptop"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["3.1.0"], "ansible_board_serial": ["DELL-LAPTOP-XPS13-001"]}</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="F25" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"]}</t>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Change product_serial and machine_id to be realistic
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2711,7 +2711,7 @@
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["nat-shared-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
@@ -2751,12 +2751,12 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["api-server-001"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL360-API"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
+          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["a644029003e46b31d1a09ecec6c77b02"], "ansible_port": [22], "ansible_product_serial": ["USE1845G8K1"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL360 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U32"], "ansible_board_serial": ["API-SERVER-001"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["e56eb592febecd4e03860514ce5a9f55"], "ansible_port": [22], "ansible_product_serial": ["USE1234567"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="H4" s="15" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["1a17f31cc8a19e2e1d3aa4901cb47939"], "ansible_port": [22], "ansible_product_serial": ["USE1234567"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
+          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["0267fc0887de14e8c994d1025a445221"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["db-primary-001"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750-DB"], "host_name": ["db-primary"]}</t>
+          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["bc2fa6de408414cef69227ebf4cf0f7e"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0DB1"], "host_name": ["db-primary"]}</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["AMD EPYC 7542 32-Core Processor"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.14.0"], "ansible_board_serial": ["DB-PRIMARY-001"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="I8" s="15" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["eddfa033379afb7784abb2e4c7dc2cf1"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
+          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["nat-shared-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
@@ -3823,12 +3823,12 @@
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["api-server-001"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL360-API"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
+          <t>{"ansible_host": ["api-server", "api-server.company.com", "api-server.company.com.east"], "ansible_machine_id": ["a644029003e46b31d1a09ecec6c77b02"], "ansible_port": [22], "ansible_product_serial": ["USE1845G8K1"], "host_name": ["api-server", "api-server.company.com", "api-server.company.com.east"]}</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_system_vendor": ["HP"], "ansible_product_name": ["ProLiant DL360 Gen10"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["HP"], "ansible_bios_version": ["U32"], "ansible_board_serial": ["API-SERVER-001"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"]}</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["machine123"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.cluster"]}</t>
+          <t>{"ansible_host": ["app01.cluster"], "ansible_machine_id": ["e56eb592febecd4e03860514ce5a9f55"], "ansible_port": [22], "ansible_product_serial": ["USE1234567"], "host_name": ["app01.cluster"]}</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["machine456"], "ansible_port": [22], "ansible_product_serial": ["HP-ProLiant-DL380"], "host_name": ["app01.failover"]}</t>
+          <t>{"ansible_host": ["app01.failover"], "ansible_machine_id": ["1a17f31cc8a19e2e1d3aa4901cb47939"], "ansible_port": [22], "ansible_product_serial": ["USE1234567"], "host_name": ["app01.failover"]}</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["ec2-synthetic-id-123"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["xyz789"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
+          <t>{"ansible_host": ["cache01.internal"], "ansible_machine_id": ["0267fc0887de14e8c994d1025a445221"], "ansible_port": [6379], "host_name": ["cache01.internal"]}</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db-cluster-node1.internal"], "ansible_machine_id": ["db-node-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R750-DB-001"], "host_name": ["db-cluster-node1.internal"]}</t>
+          <t>{"ansible_host": ["db-cluster-node1.internal"], "ansible_machine_id": ["986e14d2a7634f9bf27fa6e3e5158966"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0001"], "host_name": ["db-cluster-node1.internal"]}</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db-cluster-node2.internal"], "ansible_machine_id": ["db-node-002"], "ansible_port": [22], "ansible_product_serial": ["DELL-R750-DB-002"], "host_name": ["db-cluster-node2.internal"]}</t>
+          <t>{"ansible_host": ["db-cluster-node2.internal"], "ansible_machine_id": ["a3f70fd70db4b3daf1a0ffaec2c5d1f5"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0002"], "host_name": ["db-cluster-node2.internal"]}</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -4089,12 +4089,12 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["db-primary-001"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750-DB"], "host_name": ["db-primary"]}</t>
+          <t>{"ansible_host": ["db-primary"], "ansible_machine_id": ["bc2fa6de408414cef69227ebf4cf0f7e"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0DB1"], "host_name": ["db-primary"]}</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R750"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["AMD EPYC 7542 32-Core Processor"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.14.0"], "ansible_board_serial": ["DB-PRIMARY-001"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "db_role": ["primary"]}</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R740"], "host_name": ["db01.company.com"]}</t>
+          <t>{"ansible_host": ["db01.company.com"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0740"], "host_name": ["db01.company.com"]}</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["db02-machine-id"], "ansible_port": [22], "ansible_product_serial": ["Dell-PowerEdge-R750"], "host_name": ["db02.dev", "db02.staging"]}</t>
+          <t>{"ansible_host": ["db02.company.com"], "ansible_machine_id": ["eddfa033379afb7784abb2e4c7dc2cf1"], "ansible_port": [22], "ansible_product_serial": ["CN7016194B0750"], "host_name": ["db02.dev", "db02.staging"]}</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_machine_id": ["legacy-001"], "ansible_port": [22], "ansible_product_serial": ["HP-DL380-LEGACY-001"], "host_name": ["legacy-server.company.com"], "ansible_host": ["legacy-server.company.com"]}</t>
+          <t>{"ansible_machine_id": ["7d4afb3f5aaf1350bc54dd686568bc2d"], "ansible_port": [22], "ansible_product_serial": ["USE0123456"], "host_name": ["legacy-server.company.com"], "ansible_host": ["legacy-server.company.com"]}</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -4355,12 +4355,12 @@
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["mobile-laptop-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-LAPTOP-XPS13-001"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
+          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["797690615d609504271f6d3467fb7c7d"], "ansible_port": [22], "ansible_product_serial": ["CN0123456789"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["XPS 13 9310"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Core(TM) i7-1165G7 CPU @ 2.80GHz"], "ansible_form_factor": ["Laptop"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["3.1.0"], "ansible_board_serial": ["DELL-LAPTOP-XPS13-001"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["def789ghi012"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["web03-machine-id"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-dev-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["web04-staging-machine"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["web-backup-001", "web-primary-001"], "ansible_port": [22], "ansible_product_serial": ["DELL-R740-WEB-001", "DELL-R740-WEB-002"], "host_name": ["webserver.company.com"]}</t>
+          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["1dcd7ec391a45938c8ab4ec198a24dc5", "78a5084255b084eebb58b41f5eb85c06"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0W01", "CN7792194B0W02"], "host_name": ["webserver.company.com"]}</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["WIN-HP-DL380-001"], "host_name": ["win-srv02.company.com"]}</t>
+          <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
       <c r="F25" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Expand the data to be able to test all cases
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -671,7 +671,7 @@
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr"/>
       <c r="G7" s="8" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="n">
@@ -1794,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2037,7 +2037,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Web04 Dev Deploy</t>
+          <t>K8S Deployment Dev</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -2055,49 +2055,49 @@
         <v>1</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G8" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45846.62847222222</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45846.62847222222</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>API Server Deploy</t>
+          <t>Web04 Dev Deploy</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Development</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>45846.54166666666</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>45846.54861111111</v>
+        <v>45847.79166666666</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>AWS Instance Configuration</t>
+          <t>API Server Deploy</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -2106,28 +2106,28 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>45848.875</v>
+        <v>45846.54166666666</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>45848.87847222222</v>
+        <v>45846.54861111111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Cache Management</t>
+          <t>AWS Instance Configuration</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -2136,28 +2136,28 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>45847.59739583333</v>
+        <v>45848.875</v>
       </c>
       <c r="H11" s="16" t="n">
-        <v>45847.59739583333</v>
+        <v>45848.87847222222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Cross-Org App Deploy</t>
+          <t>Cache Management</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -2175,19 +2175,19 @@
         <v>1</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>45848.72222222222</v>
+        <v>45847.59739583333</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>45848.72222222222</v>
+        <v>45847.59739583333</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Cross-Org Web Deploy</t>
+          <t>Cross-Org App Deploy</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -2205,19 +2205,19 @@
         <v>1</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>45847.45553240741</v>
+        <v>45848.72222222222</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>45847.45553240741</v>
+        <v>45848.72222222222</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Database Backup</t>
+          <t>Cross-Org Web Deploy</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -2235,19 +2235,19 @@
         <v>1</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45847.45553240741</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>45847.56672249403</v>
+        <v>45847.45553240741</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Database Primary Deploy</t>
+          <t>Database Backup</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -2256,28 +2256,28 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>45846.58333333334</v>
+        <v>45847.56672249403</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>45846.59027777778</v>
+        <v>45847.56672249403</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Deploy Web Application</t>
+          <t>Database Primary Deploy</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -2286,28 +2286,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>45847.45207118545</v>
+        <v>45846.58333333334</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>45847.46898291037</v>
+        <v>45846.59027777778</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Log Management</t>
+          <t>Deploy Web Application</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -2322,22 +2322,22 @@
         <v>1</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="H17" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45847.46898291037</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Multi-Node App</t>
+          <t>K8S Deployment</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -2346,28 +2346,28 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G18" s="16" t="n">
-        <v>45848.70833333334</v>
+        <v>45846.625</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>45848.72916666666</v>
+        <v>45846.625</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Remote Site Management</t>
+          <t>Log Management</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -2376,28 +2376,28 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>45848.91666666666</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>45848.92013888889</v>
+        <v>45847.59062642889</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Web Deployment</t>
+          <t>Multi-Node App</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -2409,7 +2409,7 @@
         <v>2</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="15" t="n">
         <v>2</v>
@@ -2418,16 +2418,16 @@
         <v>24</v>
       </c>
       <c r="G20" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45848.70833333334</v>
       </c>
       <c r="H20" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45848.72916666666</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Web03 Deploy</t>
+          <t>Remote Site Management</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -2436,28 +2436,28 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>45847.75</v>
+        <v>45848.91666666666</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>45847.75</v>
+        <v>45848.92013888889</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Web03 Prod Deploy</t>
+          <t>Secure Host Admin</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -2475,19 +2475,19 @@
         <v>1</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G22" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45846.66666666666</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Windows Patching</t>
+          <t>Secure Host Readonly</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -2496,63 +2496,63 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="G23" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>45848.83680555555</v>
+        <v>45846.67013888889</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Staging Database Setup</t>
+          <t>Web Deployment</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="H24" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.6875</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Staging Multi-Node App</t>
+          <t>Web03 Deploy</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
@@ -2565,24 +2565,24 @@
         <v>1</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45847.75</v>
       </c>
       <c r="H25" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45847.75</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Web04 Staging Deploy</t>
+          <t>Web03 Prod Deploy</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
@@ -2598,9 +2598,129 @@
         <v>12</v>
       </c>
       <c r="G26" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>45847.75347222222</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Windows Patching</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>45848.83680555555</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Staging Database Setup</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G28" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Staging Multi-Node App</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G29" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Web04 Staging Deploy</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G30" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="H26" s="16" t="n">
+      <c r="H30" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
     </row>
@@ -2615,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3131,7 +3251,7 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>k8s-node-01.cluster</t>
         </is>
       </c>
       <c r="B13" s="15" t="n">
@@ -3141,27 +3261,27 @@
         <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45846.625</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45846.625</v>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["k8s-node-01.cluster"], "ansible_port": [22], "host_name": ["k8s-node-01.cluster"]}</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "container_runtime": ["containerd"]}</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["k8s-node-01.cluster"]</t>
         </is>
       </c>
       <c r="J13" s="15" t="n">
@@ -3171,87 +3291,87 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>k8s-node-01.internal</t>
         </is>
       </c>
       <c r="B14" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>45847.45207118545</v>
+        <v>45846.62847222222</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>45847.46898291037</v>
+        <v>45846.62847222222</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["k8s-node-01.internal"], "ansible_port": [22], "host_name": ["k8s-node-01.internal"]}</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "container_runtime": ["containerd"]}</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["k8s-node-01.internal"]</t>
         </is>
       </c>
       <c r="J14" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B15" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="J15" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>secure-host-01.company.com</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
@@ -3261,57 +3381,57 @@
         <v>2</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>45847.75</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["4f7a8b9c2d3e5f6a7b8c9d0e1f2a3b4c"], "ansible_port": [22], "ansible_product_serial": ["CN5555555555"], "host_name": ["secure-host-01.company.com"]}</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_user": ["admin", "readonly"]}</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["secure-host-01.company.com"]</t>
         </is>
       </c>
       <c r="J16" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.46898291037</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -3321,37 +3441,37 @@
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="J17" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.6875</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -3361,90 +3481,210 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45847.75</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="J19" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
+          <t>web04.dev</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>45847.79166666666</v>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="inlineStr">
+        <is>
+          <t>["web04.dev"]</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>web04.staging</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>45847.79513888889</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>45847.79513888889</v>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>["web04.staging"]</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="J22" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
           <t>win-srv02.company.com</t>
         </is>
       </c>
-      <c r="B20" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="15" t="n">
+      <c r="B23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E23" s="16" t="n">
         <v>45848.83680555555</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F23" s="16" t="n">
         <v>45848.83680555555</v>
       </c>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
+      <c r="I23" s="15" t="inlineStr">
         <is>
           <t>["win-srv02.company.com"]</t>
         </is>
       </c>
-      <c r="J20" s="15" t="n">
+      <c r="J23" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3705,7 +3945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4261,35 +4501,35 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>legacy-server.company.com</t>
+          <t>k8s-node-01.cluster</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>45846.50347222222</v>
+        <v>45846.625</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>["Development", "Production"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_machine_id": ["7d4afb3f5aaf1350bc54dd686568bc2d"], "ansible_port": [22], "ansible_product_serial": ["USE0123456"], "host_name": ["legacy-server.company.com"], "ansible_host": ["legacy-server.company.com"]}</t>
+          <t>{"ansible_host": ["k8s-node-01.cluster"], "ansible_port": [22], "host_name": ["k8s-node-01.cluster"]}</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "server_type": ["legacy"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "container_runtime": ["containerd"]}</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>["legacy-server.company.com"]</t>
+          <t>["k8s-node-01.cluster"]</t>
         </is>
       </c>
       <c r="H15" s="15" t="n">
@@ -4299,35 +4539,35 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>log01.company.com</t>
+          <t>k8s-node-01.internal</t>
         </is>
       </c>
       <c r="B16" s="16" t="n">
-        <v>45847.59069430155</v>
+        <v>45846.62847222222</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
+          <t>{"ansible_host": ["k8s-node-01.internal"], "ansible_port": [22], "host_name": ["k8s-node-01.internal"]}</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["docker"], "container_runtime": ["containerd"]}</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>["log01.company.com"]</t>
+          <t>["k8s-node-01.internal"]</t>
         </is>
       </c>
       <c r="H16" s="15" t="n">
@@ -4337,35 +4577,35 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>mobile-dev-laptop.office.company.com</t>
+          <t>legacy-server.company.com</t>
         </is>
       </c>
       <c r="B17" s="16" t="n">
-        <v>45846.375</v>
+        <v>45846.50347222222</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Development", "Production"]</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Development Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["797690615d609504271f6d3467fb7c7d"], "ansible_port": [22], "ansible_product_serial": ["CN0123456789"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
+          <t>{"ansible_machine_id": ["7d4afb3f5aaf1350bc54dd686568bc2d"], "ansible_port": [22], "ansible_product_serial": ["USE0123456"], "host_name": ["legacy-server.company.com"], "ansible_host": ["legacy-server.company.com"]}</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "server_type": ["legacy"]}</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>["mobile-dev-laptop.office.company.com"]</t>
+          <t>["legacy-server.company.com"]</t>
         </is>
       </c>
       <c r="H17" s="15" t="n">
@@ -4375,11 +4615,11 @@
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>log01.company.com</t>
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>45847.46905078303</v>
+        <v>45847.59069430155</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
@@ -4388,74 +4628,74 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["log01.company.com"], "ansible_port": [514], "host_name": ["log01.company.com"]}</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["tcp"], "ansible_virtualization_type": ["lxc"]}</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["log01.company.com"]</t>
         </is>
       </c>
       <c r="H18" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>mobile-dev-laptop.office.company.com</t>
         </is>
       </c>
       <c r="B19" s="16" t="n">
-        <v>45847.68759259259</v>
+        <v>45846.375</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["mobile-dev-laptop.office.company.com"], "ansible_machine_id": ["797690615d609504271f6d3467fb7c7d"], "ansible_port": [22], "ansible_product_serial": ["CN0123456789"], "host_name": ["mobile-dev-laptop.office.company.com"]}</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "network_context": ["office"]}</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["mobile-dev-laptop.office.company.com"]</t>
         </is>
       </c>
       <c r="H19" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>secure-host-01.company.com</t>
         </is>
       </c>
       <c r="B20" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
@@ -4464,50 +4704,50 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Production Inventory", "Restricted Inventory"]</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["4f7a8b9c2d3e5f6a7b8c9d0e1f2a3b4c"], "ansible_port": [22], "ansible_product_serial": ["CN5555555555"], "host_name": ["secure-host-01.company.com"]}</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_user": ["admin", "readonly"]}</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["secure-host-01.company.com"]</t>
         </is>
       </c>
       <c r="H20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.46905078303</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Cross-Org Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
@@ -4517,35 +4757,35 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="H21" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B22" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.68759259259</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>["Staging"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>["Staging Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
@@ -4555,21 +4795,21 @@
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="H22" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>webserver.company.com</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B23" s="16" t="n">
-        <v>45846.42013888889</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
@@ -4583,55 +4823,55 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["1dcd7ec391a45938c8ab4ec198a24dc5", "78a5084255b084eebb58b41f5eb85c06"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0W01", "CN7792194B0W02"], "host_name": ["webserver.company.com"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "server_role": ["backup", "primary"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>["webserver.company.com"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="H23" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>45846.83333333334</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["web04.dev"]</t>
         </is>
       </c>
       <c r="H24" s="15" t="n">
@@ -4641,38 +4881,152 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
+          <t>web04.staging</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>45847.79513888889</v>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>["Staging"]</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>["Staging Inventory"]</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>["web04.staging"]</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>webserver.company.com</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>45846.42013888889</v>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["1dcd7ec391a45938c8ab4ec198a24dc5", "78a5084255b084eebb58b41f5eb85c06"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0W01", "CN7792194B0W02"], "host_name": ["webserver.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "server_role": ["backup", "primary"]}</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>["webserver.company.com"]</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>45846.83333333334</v>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
           <t>win-srv02.company.com</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B28" s="16" t="n">
         <v>45846.83680555555</v>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>["Production"]</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>["Production Inventory"]</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
-      <c r="F25" s="15" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>["win-srv02.company.com"]</t>
         </is>
       </c>
-      <c r="H25" s="15" t="n">
+      <c r="H28" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4772,13 +5126,13 @@
         </is>
       </c>
       <c r="B3" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0</v>
@@ -4787,7 +5141,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -4797,13 +5151,13 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0</v>
@@ -4812,7 +5166,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Fix the NAT example
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2831,7 +2831,7 @@
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [2201, 2202], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="H2" s="15" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
+          <t>{"ansible_host": ["203.0.113.10"], "ansible_machine_id": ["639d3a53a94028d35a3f5f244793dad2"], "ansible_port": [2201, 2202], "ansible_product_serial": ["CN7792194B0NAT"], "host_name": ["nat-host-01.external", "nat-host-02.external"]}</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix case with 2 regions
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -2991,7 +2991,7 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-west"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-west"]}</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-west"]</t>
         </is>
       </c>
       <c r="J6" s="15" t="n">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-east"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-east"]}</t>
+          <t>{"ansible_host": ["aws-vm-01.us-east", "aws-vm-02.us-west"], "ansible_machine_id": ["81b0f5bd1078b9636e2a5a8f9a9e14df"], "ansible_port": [22], "ansible_product_serial": ["ec2-instance"], "host_name": ["aws-vm-01.us-east", "aws-vm-02.us-west"]}</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>["aws-vm-01.us-east", "aws-vm-02.us-east"]</t>
+          <t>["aws-vm-01.us-east", "aws-vm-02.us-west"]</t>
         </is>
       </c>
       <c r="H6" s="15" t="n">

</xml_diff>

<commit_message>
Fix test case 3.3
</commit_message>
<xml_diff>
--- a/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
+++ b/metrics_utility/test/ccspv_reports/dedup/test_complex_CCSPv2_with_canonical_facts/reports/CCSPv2-2025-07-08--2025-07-11.xlsx
@@ -671,7 +671,7 @@
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr"/>
       <c r="G7" s="8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="n">
@@ -1794,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2337,7 +2337,7 @@
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>K8S Deployment</t>
+          <t>Health Check</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -2358,16 +2358,16 @@
         <v>5</v>
       </c>
       <c r="G18" s="16" t="n">
-        <v>45846.625</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="H18" s="16" t="n">
-        <v>45846.625</v>
+        <v>45846.67013888889</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Log Management</t>
+          <t>K8S Deployment</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -2385,19 +2385,19 @@
         <v>1</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45846.625</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>45847.59062642889</v>
+        <v>45846.625</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Multi-Node App</t>
+          <t>Log Management</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -2406,28 +2406,28 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G20" s="16" t="n">
-        <v>45848.70833333334</v>
+        <v>45847.59062642889</v>
       </c>
       <c r="H20" s="16" t="n">
-        <v>45848.72916666666</v>
+        <v>45847.59062642889</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Remote Site Management</t>
+          <t>Multi-Node App</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -2439,25 +2439,25 @@
         <v>2</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>45848.91666666666</v>
+        <v>45848.70833333334</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>45848.92013888889</v>
+        <v>45848.72916666666</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>Secure Host Admin</t>
+          <t>Remote Site Management</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -2466,28 +2466,28 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G22" s="16" t="n">
-        <v>45846.66666666666</v>
+        <v>45848.91666666666</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>45846.66666666666</v>
+        <v>45848.92013888889</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Secure Host Readonly</t>
+          <t>Secure Host Admin</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -2505,19 +2505,19 @@
         <v>1</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G23" s="16" t="n">
-        <v>45846.67013888889</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>45846.67013888889</v>
+        <v>45846.66666666666</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Web Deployment</t>
+          <t>Secure Host Readonly</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
@@ -2526,28 +2526,28 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="G24" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="H24" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45846.67013888889</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Web03 Deploy</t>
+          <t>System Update</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -2565,19 +2565,19 @@
         <v>1</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>45847.75</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="H25" s="16" t="n">
-        <v>45847.75</v>
+        <v>45846.66666666666</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Web03 Prod Deploy</t>
+          <t>Web Deployment</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -2586,28 +2586,28 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.6875</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Windows Patching</t>
+          <t>Web03 Deploy</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
@@ -2616,33 +2616,33 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="15" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45847.75</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>45848.83680555555</v>
+        <v>45847.75</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Staging Database Setup</t>
+          <t>Web03 Prod Deploy</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
@@ -2655,72 +2655,132 @@
         <v>1</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G28" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="H28" s="16" t="n">
-        <v>45847.57296296296</v>
+        <v>45847.75347222222</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>Staging Multi-Node App</t>
+          <t>Windows Patching</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" s="15" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="G29" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45848.83333333334</v>
       </c>
       <c r="H29" s="16" t="n">
-        <v>45848.71527777778</v>
+        <v>45848.83680555555</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
+          <t>Staging Database Setup</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G30" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>45847.57296296296</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Staging Multi-Node App</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G31" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <v>45848.71527777778</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
           <t>Web04 Staging Deploy</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="C30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="15" t="n">
+      <c r="C32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="G30" s="16" t="n">
+      <c r="G32" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
-      <c r="H30" s="16" t="n">
+      <c r="H32" s="16" t="n">
         <v>45847.79513888889</v>
       </c>
     </row>
@@ -2735,7 +2795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3371,37 +3431,37 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>secure-host-01.company.com</t>
+          <t>secure-host-01-readonly.internal</t>
         </is>
       </c>
       <c r="B16" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>45846.66666666666</v>
+        <v>45846.67019675926</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>45846.67013888889</v>
+        <v>45846.67019675926</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["4f7a8b9c2d3e5f6a7b8c9d0e1f2a3b4c"], "ansible_port": [22], "ansible_product_serial": ["CN5555555555"], "host_name": ["secure-host-01.company.com"]}</t>
+          <t>{"ansible_host": ["secure-host-01-readonly.internal"], "ansible_machine_id": ["f8e7d6c5b4a3928170605040302010"], "ansible_port": [22], "host_name": ["secure-host-01-readonly.internal"]}</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_user": ["admin", "readonly"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "ansible_architecture": ["x86_64"]}</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>["secure-host-01.company.com"]</t>
+          <t>["secure-host-01-readonly.internal"]</t>
         </is>
       </c>
       <c r="J16" s="15" t="n">
@@ -3411,7 +3471,7 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>secure-host-01.company.com</t>
         </is>
       </c>
       <c r="B17" s="15" t="n">
@@ -3421,57 +3481,57 @@
         <v>3</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>45847.45207118545</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>45847.46898291037</v>
+        <v>45846.67013888889</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["f8e7d6c5b4a3928170605040302010"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0SEC"], "host_name": ["secure-host-01.company.com"]}</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R840"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.5.4"], "ansible_board_serial": ["CN7792194B0001"]}</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["secure-host-01.company.com"]</t>
         </is>
       </c>
       <c r="J17" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>45847.66666666666</v>
+        <v>45847.45207118545</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>45847.6875</v>
+        <v>45847.46898291037</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -3481,7 +3541,7 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
@@ -3491,7 +3551,7 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -3501,17 +3561,17 @@
         <v>2</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>45847.75</v>
+        <v>45847.66666666666</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.6875</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -3521,7 +3581,7 @@
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="J19" s="15" t="n">
@@ -3531,27 +3591,27 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.75</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
@@ -3561,17 +3621,17 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="J20" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -3581,17 +3641,17 @@
         <v>1</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -3601,7 +3661,7 @@
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["web04.dev"]</t>
         </is>
       </c>
       <c r="J21" s="15" t="n">
@@ -3611,7 +3671,7 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>web04.staging</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -3621,27 +3681,27 @@
         <v>1</v>
       </c>
       <c r="D22" s="15" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E22" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>45848.83333333334</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["web04.staging"]</t>
         </is>
       </c>
       <c r="J22" s="15" t="n">
@@ -3651,7 +3711,7 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>win-srv02.company.com</t>
+          <t>win-srv01.company.com</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -3664,27 +3724,67 @@
         <v>16</v>
       </c>
       <c r="E23" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>45848.83333333334</v>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="J23" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>win-srv02.company.com</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" s="16" t="n">
         <v>45848.83680555555</v>
       </c>
-      <c r="F23" s="16" t="n">
+      <c r="F24" s="16" t="n">
         <v>45848.83680555555</v>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I24" s="15" t="inlineStr">
         <is>
           <t>["win-srv02.company.com"]</t>
         </is>
       </c>
-      <c r="J23" s="15" t="n">
+      <c r="J24" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3945,7 +4045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4691,7 +4791,7 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>secure-host-01.company.com</t>
+          <t>secure-host-01-readonly.internal</t>
         </is>
       </c>
       <c r="B20" s="16" t="n">
@@ -4704,22 +4804,22 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory", "Restricted Inventory"]</t>
+          <t>["Restricted Inventory"]</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["4f7a8b9c2d3e5f6a7b8c9d0e1f2a3b4c"], "ansible_port": [22], "ansible_product_serial": ["CN5555555555"], "host_name": ["secure-host-01.company.com"]}</t>
+          <t>{"ansible_host": ["secure-host-01-readonly.internal"], "ansible_machine_id": ["f8e7d6c5b4a3928170605040302010"], "ansible_port": [22], "host_name": ["secure-host-01-readonly.internal"]}</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "ansible_user": ["admin", "readonly"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "ansible_architecture": ["x86_64"]}</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>["secure-host-01.company.com"]</t>
+          <t>["secure-host-01-readonly.internal"]</t>
         </is>
       </c>
       <c r="H20" s="15" t="n">
@@ -4729,11 +4829,11 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>web01.internal</t>
+          <t>secure-host-01.company.com</t>
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>45847.46905078303</v>
+        <v>45846.66666666666</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
@@ -4742,36 +4842,36 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>["Cross-Org Inventory", "Production Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
+          <t>{"ansible_host": ["secure-host-01.company.com"], "ansible_machine_id": ["f8e7d6c5b4a3928170605040302010"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0SEC"], "host_name": ["secure-host-01.company.com"]}</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["physical"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R840"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.5.4"], "ansible_board_serial": ["CN7792194B0001"]}</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>["web01.internal", "web01.prod.company.com"]</t>
+          <t>["secure-host-01.company.com"]</t>
         </is>
       </c>
       <c r="H21" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>web02.external</t>
+          <t>web01.internal</t>
         </is>
       </c>
       <c r="B22" s="16" t="n">
-        <v>45847.68759259259</v>
+        <v>45847.46905078303</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
@@ -4780,12 +4880,12 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Cross-Org Inventory", "Production Inventory"]</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
+          <t>{"ansible_host": ["web01.internal", "web01.prod.company.com"], "ansible_machine_id": ["3a2f8c9b123456789012345678901234"], "ansible_port": [22, 2222], "ansible_product_serial": ["VMware-56 4d 3a 2f 8c 9b 12 34-56 78 90 ab cd ef 12 34"], "host_name": ["web01.internal", "web01.prod.company.com"]}</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
@@ -4795,7 +4895,7 @@
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>["web02.external", "web02.internal"]</t>
+          <t>["web01.internal", "web01.prod.company.com"]</t>
         </is>
       </c>
       <c r="H22" s="15" t="n">
@@ -4805,11 +4905,11 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>web03.internal</t>
+          <t>web02.external</t>
         </is>
       </c>
       <c r="B23" s="16" t="n">
-        <v>45847.75347222222</v>
+        <v>45847.68759259259</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
@@ -4823,7 +4923,7 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
+          <t>{"ansible_host": ["web02.external", "web02.internal"], "ansible_machine_id": ["f3e2da65c5d34e59151db7ec18b868d9"], "ansible_port": [443], "ansible_product_serial": ["VMware-ab cd ef 12 34 56 78 90-12 34 56 78 90 ab cd ef"], "host_name": ["web02.external", "web02.internal"]}</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -4833,7 +4933,7 @@
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>["web03.internal", "web03.prod.internal"]</t>
+          <t>["web02.external", "web02.internal"]</t>
         </is>
       </c>
       <c r="H23" s="15" t="n">
@@ -4843,25 +4943,25 @@
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>web04.dev</t>
+          <t>web03.internal</t>
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>45847.79166666666</v>
+        <v>45847.75347222222</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>["Development"]</t>
+          <t>["Production"]</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>["Development Inventory"]</t>
+          <t>["Production Inventory"]</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
+          <t>{"ansible_host": ["web03.company.com"], "ansible_machine_id": ["01b6b28643a6a867e339e957c8ed9d37"], "ansible_port": [22, 2223], "ansible_product_serial": ["VMware-12 34 56 78 90 ab cd ef-ab cd ef 12 34 56 78 90"], "host_name": ["web03.internal", "web03.prod.internal"]}</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
@@ -4871,35 +4971,35 @@
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>["web04.dev"]</t>
+          <t>["web03.internal", "web03.prod.internal"]</t>
         </is>
       </c>
       <c r="H24" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>web04.staging</t>
+          <t>web04.dev</t>
         </is>
       </c>
       <c r="B25" s="16" t="n">
-        <v>45847.79513888889</v>
+        <v>45847.79166666666</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>["Staging"]</t>
+          <t>["Development"]</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>["Staging Inventory"]</t>
+          <t>["Development Inventory"]</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["ae920ed940e880003e264a357de969c1"], "ansible_port": [22], "ansible_product_serial": ["VMware-dev-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.dev"]}</t>
         </is>
       </c>
       <c r="F25" s="15" t="inlineStr">
@@ -4909,7 +5009,7 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>["web04.staging"]</t>
+          <t>["web04.dev"]</t>
         </is>
       </c>
       <c r="H25" s="15" t="n">
@@ -4919,35 +5019,35 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>webserver.company.com</t>
+          <t>web04.staging</t>
         </is>
       </c>
       <c r="B26" s="16" t="n">
-        <v>45846.42013888889</v>
+        <v>45847.79513888889</v>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>["Production"]</t>
+          <t>["Staging"]</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>["Production Inventory"]</t>
+          <t>["Staging Inventory"]</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["1dcd7ec391a45938c8ab4ec198a24dc5", "78a5084255b084eebb58b41f5eb85c06"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0W01", "CN7792194B0W02"], "host_name": ["webserver.company.com"]}</t>
+          <t>{"ansible_host": ["web04.company.com"], "ansible_machine_id": ["d1134fec21d571a9b596f7dbf7dc5673"], "ansible_port": [22], "ansible_product_serial": ["VMware-stg-01-02-03-04-05-06-07-08-09-10-11-12"], "host_name": ["web04.staging"]}</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "server_role": ["backup", "primary"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["VMware"], "ansible_system_vendor": ["VMware, Inc."], "ansible_product_name": ["VMware Virtual Platform"], "ansible_virtualization_role": ["guest"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Virtual"], "ansible_bios_vendor": ["Phoenix Technologies LTD"], "ansible_bios_version": ["6.00"], "ansible_board_serial": ["None"]}</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>["webserver.company.com"]</t>
+          <t>["web04.staging"]</t>
         </is>
       </c>
       <c r="H26" s="15" t="n">
@@ -4957,11 +5057,11 @@
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>win-srv01.company.com</t>
+          <t>webserver.company.com</t>
         </is>
       </c>
       <c r="B27" s="16" t="n">
-        <v>45846.83333333334</v>
+        <v>45846.42013888889</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
@@ -4975,17 +5075,17 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+          <t>{"ansible_host": ["webserver.company.com"], "ansible_machine_id": ["1dcd7ec391a45938c8ab4ec198a24dc5", "78a5084255b084eebb58b41f5eb85c06"], "ansible_port": [22], "ansible_product_serial": ["CN7792194B0W01", "CN7792194B0W02"], "host_name": ["webserver.company.com"]}</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
         <is>
-          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+          <t>{"ansible_connection_variable": ["ssh"], "ansible_virtualization_type": ["kvm"], "server_role": ["backup", "primary"]}</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>["win-srv01.company.com"]</t>
+          <t>["webserver.company.com"]</t>
         </is>
       </c>
       <c r="H27" s="15" t="n">
@@ -4995,38 +5095,76 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
+          <t>win-srv01.company.com</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>45846.83333333334</v>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>["Production"]</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>["Production Inventory"]</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_host": ["win-srv01.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv01.company.com"]}</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A88"]}</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>["win-srv01.company.com"]</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
           <t>win-srv02.company.com</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n">
+      <c r="B29" s="16" t="n">
         <v>45846.83680555555</v>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>["Production"]</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>["Production Inventory"]</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>{"ansible_host": ["win-srv02.company.com"], "ansible_port": [5985], "ansible_product_serial": ["USE9876543"], "host_name": ["win-srv02.company.com"]}</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>{"ansible_connection_variable": ["winrm"], "ansible_virtualization_type": ["VirtualPC"], "ansible_system_vendor": ["Dell Inc."], "ansible_product_name": ["PowerEdge R740"], "ansible_virtualization_role": ["host"], "ansible_architecture": ["x86_64"], "ansible_processor": ["Intel(R) Xeon(R) Gold 6248 CPU @ 2.50GHz"], "ansible_form_factor": ["Rack Mount Chassis"], "ansible_bios_vendor": ["Dell Inc."], "ansible_bios_version": ["2.13.0"], "ansible_board_serial": ["CN7792194B0A89"]}</t>
         </is>
       </c>
-      <c r="G28" s="15" t="inlineStr">
+      <c r="G29" s="15" t="inlineStr">
         <is>
           <t>["win-srv02.company.com"]</t>
         </is>
       </c>
-      <c r="H28" s="15" t="n">
+      <c r="H29" s="15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5151,13 +5289,13 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0</v>
@@ -5166,7 +5304,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>297</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5">

</xml_diff>